<commit_message>
Add transport distance computation for aviation and shipping routes
- Implemented functions to calculate great-circle routes for aviation and navigable routes for shipping.
- Introduced geocoding capabilities to resolve locations from queries.
- Added support for OSRM routing with various transport modes.
- Created a command-line interface for distance computation.
- Included error handling and response validation for external API requests.
- Established data structures for route results and waypoints.
為航空及海運路線新增運輸距離計算功能

- 實作用於計算航空大圓航線及海運可航行路線的功能。
- 導入地理編碼功能，以根據查詢結果解析位置資訊。
- 新增對多種運輸模式的 OSRM 路線規劃支援。
- 建立用於距離計算的命令列介面。
- 針對外部 API 請求加入錯誤處理與回應驗證機制。
- 建立用於儲存路線結果與航點的資料結構。
</commit_message>
<xml_diff>
--- a/resources/report_temp.xlsx
+++ b/resources/report_temp.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://accton365-my.sharepoint.com/personal/vicky_tseng_accton_com/Documents/Python/code/Excel_Vlookup_Python/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_28973FCB56869CC5CF7F1FAF523D0C4532FEDE6E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1AB8E85-831D-40FB-8ADD-628B1C7FF7AB}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_28973FCB56869CC5CF7F1FAF523D0C4532FEDE6E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{191F160E-DFAB-4D58-8BED-B17DBCC797BB}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="1284" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="1" r:id="rId1"/>
@@ -36,6 +36,9 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -786,30 +789,6 @@
   </cellStyles>
   <dxfs count="53">
     <dxf>
-      <numFmt numFmtId="13" formatCode="0%"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <condense val="0"/>
@@ -1320,19 +1299,43 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <numFmt numFmtId="13" formatCode="0%"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
@@ -7097,27 +7100,27 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="表格9" displayName="表格9" ref="B19:G24" totalsRowCount="1" headerRowDxfId="37">
   <autoFilter ref="B19:G23" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Raw Material" totalsRowFunction="custom" dataDxfId="36" totalsRowDxfId="5">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Raw Material" totalsRowFunction="custom" dataDxfId="36" totalsRowDxfId="35">
       <calculatedColumnFormula>B3/SUM(表格2[[Raw Material]:[Recycling]])</calculatedColumnFormula>
       <totalsRowFormula>SUM(B20:B23)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Manufacturing" totalsRowFunction="custom" dataDxfId="35" totalsRowDxfId="4">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Manufacturing" totalsRowFunction="custom" dataDxfId="34" totalsRowDxfId="33">
       <calculatedColumnFormula>C3/SUM(表格2[[Raw Material]:[Recycling]])</calculatedColumnFormula>
       <totalsRowFormula>SUM(C20:C23)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Distribution" totalsRowFunction="custom" dataDxfId="34" totalsRowDxfId="3">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Distribution" totalsRowFunction="custom" dataDxfId="32" totalsRowDxfId="31">
       <calculatedColumnFormula>D3/SUM(表格2[[Raw Material]:[Recycling]])</calculatedColumnFormula>
       <totalsRowFormula>SUM(D20:D23)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Usage" totalsRowFunction="custom" dataDxfId="33" totalsRowDxfId="2">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Usage" totalsRowFunction="custom" dataDxfId="30" totalsRowDxfId="29">
       <calculatedColumnFormula>E3/SUM(表格2[[Raw Material]:[Recycling]])</calculatedColumnFormula>
       <totalsRowFormula>SUM(E20:E23)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Recycling" totalsRowFunction="custom" dataDxfId="32" totalsRowDxfId="1">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Recycling" totalsRowFunction="custom" dataDxfId="28" totalsRowDxfId="27">
       <calculatedColumnFormula>F3/SUM(表格2[[Raw Material]:[Recycling]])</calculatedColumnFormula>
       <totalsRowFormula>SUM(F20:F23)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="總碳排百分比" totalsRowFunction="custom" dataDxfId="31" totalsRowDxfId="0">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="總碳排百分比" totalsRowFunction="custom" dataDxfId="26" totalsRowDxfId="25">
       <calculatedColumnFormula>SUM(B20:F20)</calculatedColumnFormula>
       <totalsRowFormula>SUM(B24:F24)</totalsRowFormula>
     </tableColumn>
@@ -7127,63 +7130,63 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="表格4" displayName="表格4" ref="A1:C11" totalsRowShown="0" headerRowBorderDxfId="30" tableBorderDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="表格4" displayName="表格4" ref="A1:C11" totalsRowShown="0" headerRowBorderDxfId="24" tableBorderDxfId="23">
   <autoFilter ref="A1:C11" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C11">
     <sortCondition descending="1" ref="C1:C11"/>
   </sortState>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="項目" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="kg CO2e" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="百分比" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="項目" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="kg CO2e" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="百分比" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="表格4_2" displayName="表格4_2" ref="A1:C11" totalsRowShown="0" headerRowBorderDxfId="25" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="表格4_2" displayName="表格4_2" ref="A1:C11" totalsRowShown="0" headerRowBorderDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="A1:C11" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="項目" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="kg CO2e" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="百分比" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="項目" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="kg CO2e" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="百分比" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="表格4_26" displayName="表格4_26" ref="A1:C11" totalsRowShown="0" headerRowBorderDxfId="20" tableBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="表格4_26" displayName="表格4_26" ref="A1:C11" totalsRowShown="0" headerRowBorderDxfId="14" tableBorderDxfId="13">
   <autoFilter ref="A1:C11" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="項目" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="kg CO2e" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="百分比" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="項目" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="kg CO2e" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="百分比" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="表格4_267" displayName="表格4_267" ref="A1:C11" totalsRowShown="0" headerRowBorderDxfId="15" tableBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="表格4_267" displayName="表格4_267" ref="A1:C11" totalsRowShown="0" headerRowBorderDxfId="9" tableBorderDxfId="8">
   <autoFilter ref="A1:C11" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="項目" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="kg CO2e" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="百分比" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="項目" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="kg CO2e" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="百分比" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="表格4_2678" displayName="表格4_2678" ref="A1:C11" totalsRowShown="0" headerRowBorderDxfId="10" tableBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="表格4_2678" displayName="表格4_2678" ref="A1:C11" totalsRowShown="0" headerRowBorderDxfId="4" tableBorderDxfId="3">
   <autoFilter ref="A1:C11" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="項目" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="kg CO2e" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="百分比" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="項目" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="kg CO2e" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="百分比" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8103,19 +8106,19 @@
         <v>0</v>
       </c>
       <c r="C7" s="51">
-        <f>SUM(C3:C5)</f>
+        <f t="shared" ref="C7:F7" si="1">SUM(C2:C5)</f>
         <v>0</v>
       </c>
       <c r="D7" s="51">
-        <f>SUM(D3:D5)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E7" s="51">
-        <f>SUM(E3:E5)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F7" s="51">
-        <f>SUM(F3:F5)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -8139,7 +8142,7 @@
         <v>0</v>
       </c>
       <c r="C11" s="4" t="e">
-        <f t="shared" ref="C11:C16" si="1">B11/B$16</f>
+        <f t="shared" ref="C11:C16" si="2">B11/B$16</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -8152,7 +8155,7 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -8165,7 +8168,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="4" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -8178,7 +8181,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="4" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -8191,7 +8194,7 @@
         <v>0</v>
       </c>
       <c r="C15" s="25" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -8204,7 +8207,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="23" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>

</xml_diff>